<commit_message>
updated sqantireads doc and scripts
</commit_message>
<xml_diff>
--- a/bankole_2026/documentation/sqanti_reads_qc_and_analysis_02ndk.xlsx
+++ b/bankole_2026/documentation/sqanti_reads_qc_and_analysis_02ndk.xlsx
@@ -841,59 +841,59 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1357,7 +1357,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="150.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>15</v>
       </c>

</xml_diff>